<commit_message>
Update 1/f ASD rows and unit-converted trial-frequency output in noise calculator
</commit_message>
<xml_diff>
--- a/solar_wind_noise/gradiometer_noise_calculator_updated_2.xlsx
+++ b/solar_wind_noise/gradiometer_noise_calculator_updated_2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lindeman\Documents\Python\gradiometer\solar_wind_noise\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lindeman\OneDrive - JPL\Documents\Python\gradiometer\solar_wind_noise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03C2699-0EEF-48D7-B123-4DA839C7582A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B2F1FE-4E49-40D4-9039-D454A7AA74EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="55935" yWindow="-1380" windowWidth="19740" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40515" yWindow="-1605" windowWidth="38700" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
   <si>
     <t>Gradiometer Noise Calculator</t>
   </si>
@@ -101,19 +101,37 @@
     <t>Sensor ASD at arithmetic band center [pT/sqrt(Hz)]</t>
   </si>
   <si>
+    <t>ratio</t>
+  </si>
+  <si>
+    <t>Arithmetic center frequency f_c,arith [Hz]</t>
+  </si>
+  <si>
     <t>Sensor ASD at geometric band center [pT/sqrt(Hz)]</t>
   </si>
   <si>
-    <t>Arithmetic center frequency f_c,arith [Hz]</t>
-  </si>
-  <si>
     <t>Geometric center frequency f_c,geom [Hz]</t>
   </si>
   <si>
+    <t>Sensor ASD at characteristic frequency [pT/sqrt(Hz)]</t>
+  </si>
+  <si>
     <t>Characteristic frequency f_char [Hz] where ASD(f_char)*sqrt(BW)=required sensor RMS</t>
   </si>
   <si>
-    <t>Sensor ASD at characteristic frequency [pT/sqrt(Hz)]</t>
+    <t>1/f ASD coefficient at 1 Hz from SQUID model [fT/sqrt(Hz)]</t>
+  </si>
+  <si>
+    <t>Integrated 1/f sensor RMS over band [pT]</t>
+  </si>
+  <si>
+    <t>Trial frequency for 1/f ASD [Hz]</t>
+  </si>
+  <si>
+    <t>1/f sensor ASD at trial frequency [pT/sqrt(Hz)]</t>
+  </si>
+  <si>
+    <t>1/f sensor ASD at trial frequency [fT/sqrt(Hz)]</t>
   </si>
   <si>
     <t>Notes:</t>
@@ -128,23 +146,30 @@
     <t>- Band center frequencies are listed below each center-ASD pair.</t>
   </si>
   <si>
-    <t>ratio</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
+    <t>- 1/f ASD model: ASD(f) = (A_1Hz/1000)/SQRT(f), where A_1Hz is in fT/sqrt(Hz) and ASD is in pT/sqrt(Hz).</t>
+  </si>
+  <si>
+    <t>- Integrated 1/f RMS over [f_low, f_high]: RMS = (A_1Hz/1000)*SQRT(LN(f_high/f_low)) [pT].</t>
+  </si>
+  <si>
+    <t>Margin factor</t>
+  </si>
+  <si>
+    <t>Maximum allowed 2/f noise at trial freq   [pT/sqrt(Hz)]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000000E+00"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -170,8 +195,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -191,6 +231,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF6F6F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -247,10 +292,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -272,12 +318,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="5" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -291,6 +343,58 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>38580</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>59448</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13573125" y="123825"/>
+          <a:ext cx="5544030" cy="4536198"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -578,101 +682,88 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="80.6640625" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="5" max="5" width="18.109375" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2">
         <v>10</v>
       </c>
-      <c r="C4" s="21">
-        <v>100000</v>
+      <c r="E4" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="2">
         <v>2</v>
       </c>
-      <c r="C5" s="2">
-        <v>2</v>
+      <c r="E5">
+        <v>1</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>8</v>
+      <c r="E6">
+        <v>2</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="18">
         <v>1</v>
       </c>
-      <c r="C7" s="18">
-        <v>1</v>
+      <c r="E7">
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>3</v>
-      </c>
-      <c r="G7">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -680,18 +771,14 @@
         <f>1/3600</f>
         <v>2.7777777777777778E-4</v>
       </c>
-      <c r="C8" s="3">
-        <f>1/3600</f>
-        <v>2.7777777777777778E-4</v>
+      <c r="E8">
+        <v>5</v>
       </c>
       <c r="F8">
-        <v>5</v>
-      </c>
-      <c r="G8">
         <v>14.444444444444439</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -699,50 +786,42 @@
         <f>1/114.483</f>
         <v>8.7349213420333145E-3</v>
       </c>
-      <c r="C9" s="3">
-        <f>1/114.483</f>
-        <v>8.7349213420333145E-3</v>
+      <c r="E9">
+        <v>7</v>
       </c>
       <c r="F9">
-        <v>7</v>
-      </c>
-      <c r="G9">
         <v>42.139999999999993</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>9</v>
+      </c>
       <c r="F10">
-        <v>9</v>
-      </c>
-      <c r="G10">
         <v>87.227392290249398</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="E11">
+        <v>11</v>
+      </c>
       <c r="F11">
-        <v>11</v>
-      </c>
-      <c r="G11">
         <v>150.95518392542391</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="10">
-        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(B5,$F$5:$F$29,$G$5:$G$29)),NA())</f>
+        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(B5,$E$5:$E$29,$F$5:$F$29)),NA())</f>
         <v>2</v>
       </c>
-      <c r="C12" s="10">
-        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(C5,$F$5:$F$29,$G$5:$G$29)),NA())</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -750,25 +829,17 @@
         <f>IF(B6="gradient",B12/(B4^2),B12)</f>
         <v>0.02</v>
       </c>
-      <c r="C13" s="5">
-        <f>IF(C6="gradient",C12/(C4^2),C12)</f>
-        <v>2.0000000000000001E-10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="19" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="12">
         <f>B7/SQRT(B13)</f>
         <v>7.0710678118654755</v>
       </c>
-      <c r="C14" s="12">
-        <f>C7/SQRT(C13)</f>
-        <v>70710.678118654745</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -776,12 +847,8 @@
         <f>B9-B8</f>
         <v>8.4571435642555367E-3</v>
       </c>
-      <c r="C15" s="5">
-        <f>C9-C8</f>
-        <v>8.4571435642555367E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -789,34 +856,27 @@
         <f>B14/SQRT(B15)</f>
         <v>76.890582439195114</v>
       </c>
-      <c r="C16" s="11">
-        <f>C14/SQRT(C15)</f>
-        <v>768905.82439195109</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="E16" t="s">
         <v>18</v>
       </c>
-      <c r="G16">
+      <c r="F16">
         <f>B16*SQRT($B$15)</f>
         <v>7.0710678118654755</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -824,16 +884,11 @@
         <f>B14^2/LN(B9/B8)</f>
         <v>14.500054993115885</v>
       </c>
-      <c r="C20" s="11">
-        <f>C14^2/LN(C9/C8)</f>
-        <v>1450005499.311588</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-    </row>
-    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -841,26 +896,22 @@
         <f>SQRT(B20/((B8+B9)/2))</f>
         <v>56.724723300480704</v>
       </c>
-      <c r="C22" s="9">
-        <f>SQRT(C20/((C8+C9)/2))</f>
-        <v>567247.23300480691</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="E22" t="s">
         <v>18</v>
       </c>
-      <c r="G22">
+      <c r="F22">
         <f>B22*SQRT($B$15)</f>
         <v>5.2165603685496462</v>
       </c>
-      <c r="I22" t="s">
-        <v>31</v>
-      </c>
-      <c r="J22">
-        <f>G22/$B$14</f>
+      <c r="H22" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22">
+        <f>F22/$B$14</f>
         <v>0.73773304221409008</v>
       </c>
     </row>
-    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -868,60 +919,46 @@
         <f>(B8+B9)/2</f>
         <v>4.5063495599055462E-3</v>
       </c>
-      <c r="C23" s="13">
-        <f>(C8+C9)/2</f>
-        <v>4.5063495599055462E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-    </row>
-    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B25" s="8">
         <f>SQRT(B20/SQRT(B8*B9))</f>
         <v>96.481867315635242</v>
       </c>
-      <c r="C25" s="8">
-        <f>SQRT(C20/SQRT(C8*C9))</f>
-        <v>964818.67315635236</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="E25" t="s">
         <v>18</v>
       </c>
-      <c r="G25">
+      <c r="F25">
         <f>B25*SQRT($B$15)</f>
         <v>8.8727358378871646</v>
       </c>
-      <c r="I25" t="s">
-        <v>31</v>
-      </c>
-      <c r="J25">
-        <f>G25/$B$14</f>
+      <c r="H25" t="s">
+        <v>22</v>
+      </c>
+      <c r="I25">
+        <f>F25/$B$14</f>
         <v>1.2547943357293836</v>
       </c>
     </row>
-    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" s="13">
         <f>SQRT(B8*B9)</f>
         <v>1.5576800183136775E-3</v>
       </c>
-      <c r="C26" s="13">
-        <f>SQRT(C8*C9)</f>
-        <v>1.5576800183136775E-3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
         <v>26</v>
       </c>
@@ -929,72 +966,147 @@
         <f>SQRT(B20/B29)</f>
         <v>76.890582439195114</v>
       </c>
-      <c r="C28" s="15">
-        <f>SQRT(C20/C29)</f>
-        <v>768905.82439195109</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="E28" t="s">
         <v>18</v>
       </c>
-      <c r="G28">
+      <c r="F28">
         <f>B28*SQRT($B$15)</f>
         <v>7.0710678118654755</v>
       </c>
       <c r="H28" t="s">
-        <v>32</v>
-      </c>
-      <c r="I28" t="s">
-        <v>31</v>
-      </c>
-      <c r="J28">
-        <f>G28/$B$14</f>
+        <v>22</v>
+      </c>
+      <c r="I28">
+        <f>F28/$B$14</f>
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B29" s="17">
         <f>B20*B15/(B14^2)</f>
         <v>2.4525809353276272E-3</v>
       </c>
-      <c r="C29" s="17">
-        <f>C20*C15/(C14^2)</f>
-        <v>2.4525809353276272E-3</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="E29" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
+      <c r="B31" s="20">
+        <v>22.5167</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
+      <c r="B32" s="26">
+        <f>SQRT((B31/1000)^2*LN(B9/B8))</f>
+        <v>4.1812382921966061E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="23"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
         <v>30</v>
       </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="21">
+        <f>(B31/1000)/SQRT(B34)</f>
+        <v>2.2516700000000001E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" s="20">
+        <f>1000*B35</f>
+        <v>22.5167</v>
+      </c>
+      <c r="C36" s="20"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="22">
+        <f>B14/B32</f>
+        <v>169.11420296379958</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="27">
+        <f>B35*B38</f>
+        <v>3.8078937738749863</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="4"/>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>